<commit_message>
Update column name for plant capacity in solar analytics
</commit_message>
<xml_diff>
--- a/orchestrator/masters/Solar_installation.xlsx
+++ b/orchestrator/masters/Solar_installation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/HPCL_INFRA/dnc_backend_v2/orchestrator/masters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA27A7C9-C44D-E749-B8EF-F95D965DD0B0}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8587A661-732C-8945-92AA-E6ECC1724000}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,10 +31,6 @@
     <t>Location</t>
   </si>
   <si>
-    <t>Plant Capacity
-  KWp</t>
-  </si>
-  <si>
     <t>DOC</t>
   </si>
   <si>
@@ -657,6 +653,9 @@
   </si>
   <si>
     <t>1937/Suryapet Terminal/400KWp/Set-2</t>
+  </si>
+  <si>
+    <t>Plant Capacity  KWp</t>
   </si>
 </sst>
 </file>
@@ -664,9 +663,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -678,6 +677,12 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF54B33E"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -715,12 +720,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1042,7 +1048,7 @@
     <col min="14" max="14" width="12.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:14" ht="16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1052,49 +1058,49 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>1305</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D2">
         <v>12</v>
@@ -1103,7 +1109,7 @@
         <v>42381</v>
       </c>
       <c r="F2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G2">
         <v>1440</v>
@@ -1115,10 +1121,10 @@
         <v>93.115635500529038</v>
       </c>
       <c r="J2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L2">
         <v>10778.32104045724</v>
@@ -1132,13 +1138,13 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3">
         <v>1281</v>
       </c>
       <c r="C3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3">
         <v>15</v>
@@ -1147,7 +1153,7 @@
         <v>42739</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G3">
         <v>1800</v>
@@ -1159,10 +1165,10 @@
         <v>93.759407787967987</v>
       </c>
       <c r="J3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L3">
         <v>10238.527330446101</v>
@@ -1176,13 +1182,13 @@
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B4">
         <v>1999</v>
       </c>
       <c r="C4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4">
         <v>550</v>
@@ -1191,7 +1197,7 @@
         <v>45302</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G4">
         <v>66000</v>
@@ -1203,10 +1209,10 @@
         <v>99</v>
       </c>
       <c r="J4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L4">
         <v>396396</v>
@@ -1220,13 +1226,13 @@
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B5">
         <v>1221</v>
       </c>
       <c r="C5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D5">
         <v>850</v>
@@ -1235,7 +1241,7 @@
         <v>45560</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G5">
         <v>102000</v>
@@ -1247,10 +1253,10 @@
         <v>99</v>
       </c>
       <c r="J5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L5">
         <v>765765</v>
@@ -1264,13 +1270,13 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6">
         <v>1305</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6">
         <v>120</v>
@@ -1279,7 +1285,7 @@
         <v>44651</v>
       </c>
       <c r="F6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G6">
         <v>14400</v>
@@ -1291,10 +1297,10 @@
         <v>97.273776836918415</v>
       </c>
       <c r="J6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L6">
         <v>84978.371444731936</v>
@@ -1308,13 +1314,13 @@
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7">
         <v>1879</v>
       </c>
       <c r="C7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D7">
         <v>20</v>
@@ -1323,7 +1329,7 @@
         <v>43237</v>
       </c>
       <c r="F7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G7">
         <v>2400</v>
@@ -1335,10 +1341,10 @@
         <v>94.662343263744077</v>
       </c>
       <c r="J7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L7">
         <v>13782.83717920114</v>
@@ -1352,13 +1358,13 @@
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8">
         <v>1128</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D8">
         <v>25</v>
@@ -1367,7 +1373,7 @@
         <v>42820</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G8">
         <v>3000</v>
@@ -1379,10 +1385,10 @@
         <v>93.905682106953321</v>
       </c>
       <c r="J8" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L8">
         <v>17090.834143465501</v>
@@ -1396,13 +1402,13 @@
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>1856</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D9">
         <v>60</v>
@@ -1411,7 +1417,7 @@
         <v>43318</v>
       </c>
       <c r="F9" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G9">
         <v>7200</v>
@@ -1423,10 +1429,10 @@
         <v>94.810026254935451</v>
       </c>
       <c r="J9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K9" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L9">
         <v>41413.019468155813</v>
@@ -1440,13 +1446,13 @@
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B10">
         <v>1979</v>
       </c>
       <c r="C10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D10">
         <v>130</v>
@@ -1455,7 +1461,7 @@
         <v>43619</v>
       </c>
       <c r="F10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G10">
         <v>15600</v>
@@ -1467,10 +1473,10 @@
         <v>95.360845290742347</v>
       </c>
       <c r="J10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L10">
         <v>90249.50398315856</v>
@@ -1484,13 +1490,13 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B11">
         <v>1242</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D11">
         <v>15</v>
@@ -1499,7 +1505,7 @@
         <v>42739</v>
       </c>
       <c r="F11" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G11">
         <v>1800</v>
@@ -1511,10 +1517,10 @@
         <v>93.759407787967987</v>
       </c>
       <c r="J11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L11">
         <v>11518.343246751871</v>
@@ -1528,13 +1534,13 @@
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B12">
         <v>1242</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D12">
         <v>50</v>
@@ -1543,7 +1549,7 @@
         <v>45292</v>
       </c>
       <c r="F12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G12">
         <v>6000</v>
@@ -1555,10 +1561,10 @@
         <v>99</v>
       </c>
       <c r="J12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L12">
         <v>36036</v>
@@ -1572,13 +1578,13 @@
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>1334</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D13">
         <v>15</v>
@@ -1587,7 +1593,7 @@
         <v>42576</v>
       </c>
       <c r="F13" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G13">
         <v>1800</v>
@@ -1599,10 +1605,10 @@
         <v>93.465743523452247</v>
       </c>
       <c r="J13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L13">
         <v>10206.459192760991</v>
@@ -1616,13 +1622,13 @@
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B14">
         <v>1278</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D14">
         <v>350</v>
@@ -1631,7 +1637,7 @@
         <v>42739</v>
       </c>
       <c r="F14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G14">
         <v>42000</v>
@@ -1643,10 +1649,10 @@
         <v>93.759407787967987</v>
       </c>
       <c r="J14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L14">
         <v>238898.97104374241</v>
@@ -1660,13 +1666,13 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B15">
         <v>1940</v>
       </c>
       <c r="C15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D15">
         <v>150</v>
@@ -1675,7 +1681,7 @@
         <v>45382</v>
       </c>
       <c r="F15" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G15">
         <v>18000</v>
@@ -1687,10 +1693,10 @@
         <v>99</v>
       </c>
       <c r="J15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L15">
         <v>108108</v>
@@ -1704,13 +1710,13 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B16">
         <v>1940</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D16">
         <v>102</v>
@@ -1719,7 +1725,7 @@
         <v>43524</v>
       </c>
       <c r="F16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G16">
         <v>12240</v>
@@ -1731,10 +1737,10 @@
         <v>95.186654014699883</v>
       </c>
       <c r="J16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L16">
         <v>70681.801805155541</v>
@@ -1748,13 +1754,13 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B17">
         <v>1221</v>
       </c>
       <c r="C17" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D17">
         <v>64</v>
@@ -1763,7 +1769,7 @@
         <v>42691</v>
       </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G17">
         <v>7680</v>
@@ -1775,10 +1781,10 @@
         <v>93.672834249330094</v>
       </c>
       <c r="J17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L17">
         <v>43644.046933447877</v>
@@ -1792,13 +1798,13 @@
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B18">
         <v>1953</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D18">
         <v>130</v>
@@ -1807,7 +1813,7 @@
         <v>43518</v>
       </c>
       <c r="F18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G18">
         <v>15600</v>
@@ -1819,10 +1825,10 @@
         <v>95.175663149151134</v>
       </c>
       <c r="J18" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K18" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L18">
         <v>90074.247604356628</v>
@@ -1836,13 +1842,13 @@
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B19">
         <v>1919</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D19">
         <v>177</v>
@@ -1851,7 +1857,7 @@
         <v>43105</v>
       </c>
       <c r="F19" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G19">
         <v>21240</v>
@@ -1863,10 +1869,10 @@
         <v>94.422167425906181</v>
       </c>
       <c r="J19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K19" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L19">
         <v>121668.6280583257</v>
@@ -1880,13 +1886,13 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B20">
         <v>1341</v>
       </c>
       <c r="C20" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D20">
         <v>265</v>
@@ -1895,7 +1901,7 @@
         <v>45016</v>
       </c>
       <c r="F20" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G20">
         <v>31800</v>
@@ -1907,10 +1913,10 @@
         <v>99</v>
       </c>
       <c r="J20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L20">
         <v>190990.8</v>
@@ -1924,13 +1930,13 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B21">
         <v>1385</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D21">
         <v>56</v>
@@ -1939,7 +1945,7 @@
         <v>43104</v>
       </c>
       <c r="F21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G21">
         <v>6720</v>
@@ -1951,10 +1957,10 @@
         <v>94.420350239645515</v>
       </c>
       <c r="J21" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L21">
         <v>38493.288385698681</v>
@@ -1968,13 +1974,13 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B22">
         <v>1644</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D22">
         <v>37</v>
@@ -1983,7 +1989,7 @@
         <v>42292</v>
       </c>
       <c r="F22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G22">
         <v>4440</v>
@@ -1995,10 +2001,10 @@
         <v>92.956278778110672</v>
       </c>
       <c r="J22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K22" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L22">
         <v>25038.70325167189</v>
@@ -2012,13 +2018,13 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B23">
         <v>1504</v>
       </c>
       <c r="C23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D23">
         <v>80</v>
@@ -2027,7 +2033,7 @@
         <v>45565</v>
       </c>
       <c r="F23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G23">
         <v>9600</v>
@@ -2039,10 +2045,10 @@
         <v>99</v>
       </c>
       <c r="J23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K23" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L23">
         <v>57657.599999999999</v>
@@ -2056,13 +2062,13 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B24">
         <v>1485</v>
       </c>
       <c r="C24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D24">
         <v>75</v>
@@ -2071,7 +2077,7 @@
         <v>43468</v>
       </c>
       <c r="F24" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G24">
         <v>9000</v>
@@ -2083,10 +2089,10 @@
         <v>95.084121941950855</v>
       </c>
       <c r="J24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L24">
         <v>51915.930580305168</v>
@@ -2100,13 +2106,13 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B25">
         <v>1410</v>
       </c>
       <c r="C25" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D25">
         <v>613</v>
@@ -2115,7 +2121,7 @@
         <v>45046</v>
       </c>
       <c r="F25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G25">
         <v>73560</v>
@@ -2127,10 +2133,10 @@
         <v>99</v>
       </c>
       <c r="J25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L25">
         <v>441801.36</v>
@@ -2144,13 +2150,13 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B26">
         <v>1146</v>
       </c>
       <c r="C26" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D26">
         <v>25</v>
@@ -2159,7 +2165,7 @@
         <v>45126</v>
       </c>
       <c r="F26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G26">
         <v>3000</v>
@@ -2171,10 +2177,10 @@
         <v>99</v>
       </c>
       <c r="J26" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L26">
         <v>18018</v>
@@ -2188,13 +2194,13 @@
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B27">
         <v>1313</v>
       </c>
       <c r="C27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D27">
         <v>25</v>
@@ -2203,7 +2209,7 @@
         <v>43253</v>
       </c>
       <c r="F27" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G27">
         <v>3000</v>
@@ -2215,10 +2221,10 @@
         <v>94.691496969036365</v>
       </c>
       <c r="J27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K27" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L27">
         <v>17233.852448364622</v>
@@ -2232,13 +2238,13 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B28">
         <v>1991</v>
       </c>
       <c r="C28" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D28">
         <v>120</v>
@@ -2247,7 +2253,7 @@
         <v>43362</v>
       </c>
       <c r="F28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="G28">
         <v>14400</v>
@@ -2259,10 +2265,10 @@
         <v>94.890345662340223</v>
       </c>
       <c r="J28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L28">
         <v>82896.205970620416</v>
@@ -2276,13 +2282,13 @@
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B29">
         <v>1254</v>
       </c>
       <c r="C29" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D29">
         <v>20</v>
@@ -2291,7 +2297,7 @@
         <v>42576</v>
       </c>
       <c r="F29" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G29">
         <v>2400</v>
@@ -2303,10 +2309,10 @@
         <v>93.465743523452247</v>
       </c>
       <c r="J29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L29">
         <v>13608.612257014651</v>
@@ -2320,13 +2326,13 @@
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B30">
         <v>1457</v>
       </c>
       <c r="C30" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D30">
         <v>100</v>
@@ -2335,7 +2341,7 @@
         <v>45077</v>
       </c>
       <c r="F30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="G30">
         <v>12000</v>
@@ -2347,10 +2353,10 @@
         <v>99</v>
       </c>
       <c r="J30" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K30" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L30">
         <v>72072</v>
@@ -2364,13 +2370,13 @@
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B31">
         <v>1777</v>
       </c>
       <c r="C31" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D31">
         <v>81</v>
@@ -2379,7 +2385,7 @@
         <v>43467</v>
       </c>
       <c r="F31" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G31">
         <v>9720</v>
@@ -2391,10 +2397,10 @@
         <v>95.082292016153659</v>
       </c>
       <c r="J31" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K31" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L31">
         <v>56068.125956085489</v>
@@ -2408,13 +2414,13 @@
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B32">
         <v>1292</v>
       </c>
       <c r="C32" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D32">
         <v>25</v>
@@ -2423,7 +2429,7 @@
         <v>42824</v>
       </c>
       <c r="F32" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="G32">
         <v>3000</v>
@@ -2435,10 +2441,10 @@
         <v>93.912911440087655</v>
       </c>
       <c r="J32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K32" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L32">
         <v>17092.14988209595</v>
@@ -2452,13 +2458,13 @@
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B33">
         <v>1937</v>
       </c>
       <c r="C33" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D33">
         <v>81</v>
@@ -2467,7 +2473,7 @@
         <v>43605</v>
       </c>
       <c r="F33" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G33">
         <v>9720</v>
@@ -2479,10 +2485,10 @@
         <v>95.335154984586325</v>
       </c>
       <c r="J33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K33" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L33">
         <v>56217.234191310861</v>
@@ -2496,13 +2502,13 @@
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B34">
         <v>1991</v>
       </c>
       <c r="C34" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D34">
         <v>250</v>
@@ -2511,7 +2517,7 @@
         <v>43552</v>
       </c>
       <c r="F34" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G34">
         <v>30000</v>
@@ -2523,10 +2529,10 @@
         <v>95.237961504909336</v>
       </c>
       <c r="J34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K34" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L34">
         <v>173333.08993893501</v>
@@ -2540,13 +2546,13 @@
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B35">
         <v>1436</v>
       </c>
       <c r="C35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D35">
         <v>25</v>
@@ -2555,7 +2561,7 @@
         <v>43154</v>
       </c>
       <c r="F35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="G35">
         <v>3000</v>
@@ -2567,10 +2573,10 @@
         <v>94.511252407838072</v>
       </c>
       <c r="J35" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K35" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L35">
         <v>17201.047938226529</v>
@@ -2584,13 +2590,13 @@
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B36">
         <v>3718</v>
       </c>
       <c r="C36" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D36">
         <v>81.2</v>
@@ -2599,7 +2605,7 @@
         <v>43467</v>
       </c>
       <c r="F36" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G36">
         <v>9744</v>
@@ -2611,10 +2617,10 @@
         <v>95.082292016153659</v>
       </c>
       <c r="J36" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K36" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L36">
         <v>56206.565773261013</v>
@@ -2628,13 +2634,13 @@
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B37">
         <v>1583</v>
       </c>
       <c r="C37" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D37">
         <v>33</v>
@@ -2643,7 +2649,7 @@
         <v>43469</v>
       </c>
       <c r="F37" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G37">
         <v>3960</v>
@@ -2655,10 +2661,10 @@
         <v>95.085951902966272</v>
       </c>
       <c r="J37" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L37">
         <v>22843.44908516861</v>
@@ -2672,13 +2678,13 @@
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B38">
         <v>1216</v>
       </c>
       <c r="C38" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D38">
         <v>750</v>
@@ -2687,7 +2693,7 @@
         <v>43091</v>
       </c>
       <c r="F38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="G38">
         <v>90000</v>
@@ -2699,10 +2705,10 @@
         <v>94.396730000496504</v>
       </c>
       <c r="J38" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K38" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L38">
         <v>515406.1458027109</v>
@@ -2716,13 +2722,13 @@
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B39">
         <v>1723</v>
       </c>
       <c r="C39" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D39">
         <v>240</v>
@@ -2731,7 +2737,7 @@
         <v>43832</v>
       </c>
       <c r="F39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="G39">
         <v>28800</v>
@@ -2743,10 +2749,10 @@
         <v>95.752559935703587</v>
       </c>
       <c r="J39" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K39" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L39">
         <v>167298.8727196613</v>
@@ -2760,13 +2766,13 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B40">
         <v>1800</v>
       </c>
       <c r="C40" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D40">
         <v>40.6</v>
@@ -2775,7 +2781,7 @@
         <v>43570</v>
       </c>
       <c r="F40" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="G40">
         <v>4872</v>
@@ -2787,10 +2793,10 @@
         <v>95.270959494466183</v>
       </c>
       <c r="J40" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K40" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L40">
         <v>28159.04695586038</v>
@@ -2804,13 +2810,13 @@
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B41">
         <v>1334</v>
       </c>
       <c r="C41" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D41">
         <v>75</v>
@@ -2819,7 +2825,7 @@
         <v>43334</v>
       </c>
       <c r="F41" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="G41">
         <v>9000</v>
@@ -2831,10 +2837,10 @@
         <v>94.839225443006342</v>
       </c>
       <c r="J41" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L41">
         <v>51782.217091881474</v>
@@ -2848,13 +2854,13 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B42">
         <v>1305</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D42">
         <v>7.5</v>
@@ -2863,7 +2869,7 @@
         <v>42008</v>
       </c>
       <c r="F42" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="G42">
         <v>900</v>
@@ -2875,10 +2881,10 @@
         <v>92.449591032308831</v>
       </c>
       <c r="J42" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K42" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L42">
         <v>5047.7476703640623</v>
@@ -2892,13 +2898,13 @@
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B43">
         <v>1292</v>
       </c>
       <c r="C43" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D43">
         <v>44.3</v>
@@ -2907,7 +2913,7 @@
         <v>44098</v>
       </c>
       <c r="F43" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="G43">
         <v>5316</v>
@@ -2919,10 +2925,10 @@
         <v>96.244003674752122</v>
       </c>
       <c r="J43" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K43" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L43">
         <v>31039.076161122259</v>
@@ -2936,13 +2942,13 @@
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B44">
         <v>1871</v>
       </c>
       <c r="C44" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D44">
         <v>75</v>
@@ -2951,7 +2957,7 @@
         <v>43425</v>
       </c>
       <c r="F44" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G44">
         <v>9000</v>
@@ -2963,10 +2969,10 @@
         <v>95.005466925742752</v>
       </c>
       <c r="J44" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K44" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L44">
         <v>51872.984941455543</v>
@@ -2980,13 +2986,13 @@
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B45">
         <v>1436</v>
       </c>
       <c r="C45" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D45">
         <v>75</v>
@@ -2995,7 +3001,7 @@
         <v>45016</v>
       </c>
       <c r="F45" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="G45">
         <v>9000</v>
@@ -3007,10 +3013,10 @@
         <v>99</v>
       </c>
       <c r="J45" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K45" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L45">
         <v>54054</v>
@@ -3024,13 +3030,13 @@
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B46">
         <v>1919</v>
       </c>
       <c r="C46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D46">
         <v>75</v>
@@ -3039,7 +3045,7 @@
         <v>43105</v>
       </c>
       <c r="F46" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G46">
         <v>9000</v>
@@ -3051,10 +3057,10 @@
         <v>94.422167425906181</v>
       </c>
       <c r="J46" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K46" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L46">
         <v>51554.503414544772</v>
@@ -3068,13 +3074,13 @@
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B47">
         <v>1233</v>
       </c>
       <c r="C47" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D47">
         <v>138</v>
@@ -3083,7 +3089,7 @@
         <v>42739</v>
       </c>
       <c r="F47" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G47">
         <v>16560</v>
@@ -3095,10 +3101,10 @@
         <v>93.759407787967987</v>
       </c>
       <c r="J47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K47" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L47">
         <v>94194.451440104152</v>
@@ -3112,13 +3118,13 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B48">
         <v>1584</v>
       </c>
       <c r="C48" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D48">
         <v>10</v>
@@ -3127,7 +3133,7 @@
         <v>42739</v>
       </c>
       <c r="F48" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="G48">
         <v>1200</v>
@@ -3139,10 +3145,10 @@
         <v>93.759407787967987</v>
       </c>
       <c r="J48" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K48" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L48">
         <v>6825.6848869640698</v>
@@ -3156,13 +3162,13 @@
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B49">
         <v>1636</v>
       </c>
       <c r="C49" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D49">
         <v>30</v>
@@ -3171,7 +3177,7 @@
         <v>43107</v>
       </c>
       <c r="F49" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G49">
         <v>3600</v>
@@ -3183,10 +3189,10 @@
         <v>94.425801903347278</v>
       </c>
       <c r="J49" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K49" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L49">
         <v>20622.595135691041</v>
@@ -3200,13 +3206,13 @@
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B50">
         <v>1485</v>
       </c>
       <c r="C50" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D50">
         <v>75</v>
@@ -3215,7 +3221,7 @@
         <v>45272</v>
       </c>
       <c r="F50" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G50">
         <v>9000</v>
@@ -3227,10 +3233,10 @@
         <v>99</v>
       </c>
       <c r="J50" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K50" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L50">
         <v>54054</v>
@@ -3244,13 +3250,13 @@
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B51">
         <v>1265</v>
       </c>
       <c r="C51" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D51">
         <v>16</v>
@@ -3259,7 +3265,7 @@
         <v>43769</v>
       </c>
       <c r="F51" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="G51">
         <v>1920</v>
@@ -3271,10 +3277,10 @@
         <v>95.636533395015761</v>
       </c>
       <c r="J51" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K51" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L51">
         <v>11139.74340985143</v>
@@ -3288,13 +3294,13 @@
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B52">
         <v>1723</v>
       </c>
       <c r="C52" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D52">
         <v>55</v>
@@ -3303,7 +3309,7 @@
         <v>43106</v>
       </c>
       <c r="F52" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G52">
         <v>6600</v>
@@ -3315,10 +3321,10 @@
         <v>94.423984647139875</v>
       </c>
       <c r="J52" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K52" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L52">
         <v>37807.36345271481</v>
@@ -3332,13 +3338,13 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B53">
         <v>1265</v>
       </c>
       <c r="C53" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D53">
         <v>4</v>
@@ -3347,7 +3353,7 @@
         <v>43769</v>
       </c>
       <c r="F53" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G53">
         <v>480</v>
@@ -3359,10 +3365,10 @@
         <v>95.636533395015761</v>
       </c>
       <c r="J53" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K53" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L53">
         <v>2784.9358524628592</v>
@@ -3376,13 +3382,13 @@
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B54">
         <v>1845</v>
       </c>
       <c r="C54" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D54">
         <v>65</v>
@@ -3391,7 +3397,7 @@
         <v>43474</v>
       </c>
       <c r="F54" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="G54">
         <v>7800</v>
@@ -3403,10 +3409,10 @@
         <v>95.095102236340267</v>
       </c>
       <c r="J54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K54" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L54">
         <v>44999.002378236211</v>
@@ -3420,13 +3426,13 @@
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B55">
         <v>1797</v>
       </c>
       <c r="C55" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D55">
         <v>39</v>
@@ -3435,7 +3441,7 @@
         <v>43577</v>
       </c>
       <c r="F55" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="G55">
         <v>4680</v>
@@ -3447,10 +3453,10 @@
         <v>95.283795133391536</v>
       </c>
       <c r="J55" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K55" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L55">
         <v>27052.975114272529</v>
@@ -3464,13 +3470,13 @@
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B56">
         <v>1656</v>
       </c>
       <c r="C56" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D56">
         <v>60</v>
@@ -3479,7 +3485,7 @@
         <v>43110</v>
       </c>
       <c r="F56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G56">
         <v>7200</v>
@@ -3491,10 +3497,10 @@
         <v>94.431253881818435</v>
       </c>
       <c r="J56" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K56" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L56">
         <v>41247.571695578292</v>
@@ -3508,13 +3514,13 @@
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B57">
         <v>1509</v>
       </c>
       <c r="C57" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D57">
         <v>45</v>
@@ -3523,7 +3529,7 @@
         <v>43604</v>
       </c>
       <c r="F57" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="G57">
         <v>5400</v>
@@ -3535,10 +3541,10 @@
         <v>95.333320227574077</v>
       </c>
       <c r="J57" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K57" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L57">
         <v>31231.19570655327</v>
@@ -3552,13 +3558,13 @@
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B58">
         <v>1292</v>
       </c>
       <c r="C58" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D58">
         <v>19.8</v>
@@ -3567,7 +3573,7 @@
         <v>43890</v>
       </c>
       <c r="F58" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G58">
         <v>2376</v>
@@ -3579,10 +3585,10 @@
         <v>95.859502466281356</v>
       </c>
       <c r="J58" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K58" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L58">
         <v>13817.57212349966</v>
@@ -3596,13 +3602,13 @@
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B59">
         <v>1583</v>
       </c>
       <c r="C59" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D59">
         <v>150</v>
@@ -3611,7 +3617,7 @@
         <v>45107</v>
       </c>
       <c r="F59" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="G59">
         <v>18000</v>
@@ -3623,10 +3629,10 @@
         <v>99</v>
       </c>
       <c r="J59" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K59" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L59">
         <v>108108</v>
@@ -3640,13 +3646,13 @@
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B60">
         <v>1723</v>
       </c>
       <c r="C60" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D60">
         <v>200</v>
@@ -3655,7 +3661,7 @@
         <v>43106</v>
       </c>
       <c r="F60" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G60">
         <v>24000</v>
@@ -3667,10 +3673,10 @@
         <v>94.423984647139875</v>
       </c>
       <c r="J60" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K60" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L60">
         <v>137481.32164623571</v>
@@ -3684,13 +3690,13 @@
     </row>
     <row r="61" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B61">
         <v>1895</v>
       </c>
       <c r="C61" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D61">
         <v>158.27500000000001</v>
@@ -3699,7 +3705,7 @@
         <v>43489</v>
       </c>
       <c r="F61" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G61">
         <v>18993</v>
@@ -3711,10 +3717,10 @@
         <v>95.122558520143244</v>
       </c>
       <c r="J61" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K61" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L61">
         <v>109604.2070743669</v>
@@ -3728,13 +3734,13 @@
     </row>
     <row r="62" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B62">
         <v>1504</v>
       </c>
       <c r="C62" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D62">
         <v>30</v>
@@ -3743,7 +3749,7 @@
         <v>43802</v>
       </c>
       <c r="F62" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="G62">
         <v>3600</v>
@@ -3755,10 +3761,10 @@
         <v>95.697291656943932</v>
       </c>
       <c r="J62" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K62" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L62">
         <v>20900.288497876551</v>
@@ -3772,13 +3778,13 @@
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B63">
         <v>1183</v>
       </c>
       <c r="C63" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D63">
         <v>40</v>
@@ -3787,7 +3793,7 @@
         <v>43131</v>
       </c>
       <c r="F63" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="G63">
         <v>4800</v>
@@ -3799,10 +3805,10 @@
         <v>94.469426546186625</v>
       </c>
       <c r="J63" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K63" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L63">
         <v>27509.49701024955</v>
@@ -3816,13 +3822,13 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B64">
         <v>1157</v>
       </c>
       <c r="C64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D64">
         <v>50</v>
@@ -3831,7 +3837,7 @@
         <v>43106</v>
       </c>
       <c r="F64" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="G64">
         <v>6000</v>
@@ -3843,10 +3849,10 @@
         <v>94.423984647139875</v>
       </c>
       <c r="J64" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K64" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L64">
         <v>34370.330411558913</v>
@@ -3860,13 +3866,13 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B65">
         <v>1630</v>
       </c>
       <c r="C65" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="D65">
         <v>100</v>
@@ -3875,7 +3881,7 @@
         <v>43880</v>
       </c>
       <c r="F65" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G65">
         <v>12000</v>
@@ -3887,10 +3893,10 @@
         <v>95.841055581359029</v>
       </c>
       <c r="J65" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K65" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L65">
         <v>69772.288463229372</v>
@@ -3904,13 +3910,13 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B66">
         <v>1712</v>
       </c>
       <c r="C66" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D66">
         <v>30</v>
@@ -3919,7 +3925,7 @@
         <v>43102</v>
       </c>
       <c r="F66" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="G66">
         <v>3600</v>
@@ -3931,10 +3937,10 @@
         <v>94.416715972040578</v>
       </c>
       <c r="J66" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K66" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L66">
         <v>20620.61076829366</v>
@@ -3948,13 +3954,13 @@
     </row>
     <row r="67" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B67">
         <v>1128</v>
       </c>
       <c r="C67" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D67">
         <v>15</v>
@@ -3963,7 +3969,7 @@
         <v>42820</v>
       </c>
       <c r="F67" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G67">
         <v>1800</v>
@@ -3975,10 +3981,10 @@
         <v>93.905682106953321</v>
       </c>
       <c r="J67" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K67" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L67">
         <v>10254.5004860793</v>
@@ -3992,13 +3998,13 @@
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B68">
         <v>1584</v>
       </c>
       <c r="C68" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D68">
         <v>40</v>
@@ -4007,7 +4013,7 @@
         <v>42903</v>
       </c>
       <c r="F68" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="G68">
         <v>4800</v>
@@ -4019,10 +4025,10 @@
         <v>94.055804865064175</v>
       </c>
       <c r="J68" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K68" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L68">
         <v>27389.050376706691</v>
@@ -4036,13 +4042,13 @@
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B69">
         <v>1435</v>
       </c>
       <c r="C69" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D69">
         <v>100</v>
@@ -4051,7 +4057,7 @@
         <v>43372</v>
       </c>
       <c r="F69" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="G69">
         <v>12000</v>
@@ -4063,10 +4069,10 @@
         <v>94.908609560583571</v>
       </c>
       <c r="J69" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K69" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L69">
         <v>69093.467760104832</v>
@@ -4080,13 +4086,13 @@
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B70">
         <v>1504</v>
       </c>
       <c r="C70" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D70">
         <v>65</v>
@@ -4095,7 +4101,7 @@
         <v>45296</v>
       </c>
       <c r="F70" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G70">
         <v>7800</v>
@@ -4107,10 +4113,10 @@
         <v>99</v>
       </c>
       <c r="J70" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K70" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L70">
         <v>46846.8</v>
@@ -4124,13 +4130,13 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B71">
         <v>1915</v>
       </c>
       <c r="C71" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D71">
         <v>39</v>
@@ -4139,7 +4145,7 @@
         <v>43783</v>
       </c>
       <c r="F71" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G71">
         <v>4680</v>
@@ -4151,10 +4157,10 @@
         <v>95.662304914692996</v>
       </c>
       <c r="J71" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K71" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L71">
         <v>27160.44161137964</v>
@@ -4168,13 +4174,13 @@
     </row>
     <row r="72" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B72">
         <v>1992</v>
       </c>
       <c r="C72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D72">
         <v>1000</v>
@@ -4183,7 +4189,7 @@
         <v>43370</v>
       </c>
       <c r="F72" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="G72">
         <v>120000</v>
@@ -4195,10 +4201,10 @@
         <v>94.904956499730901</v>
       </c>
       <c r="J72" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K72" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L72">
         <v>690908.08331804094</v>
@@ -4212,13 +4218,13 @@
     </row>
     <row r="73" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B73">
         <v>1319</v>
       </c>
       <c r="C73" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D73">
         <v>125</v>
@@ -4227,7 +4233,7 @@
         <v>43403</v>
       </c>
       <c r="F73" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G73">
         <v>15000</v>
@@ -4239,10 +4245,10 @@
         <v>94.965249988009859</v>
       </c>
       <c r="J73" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K73" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L73">
         <v>86418.377489088976</v>
@@ -4256,13 +4262,13 @@
     </row>
     <row r="74" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B74">
         <v>1991</v>
       </c>
       <c r="C74" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D74">
         <v>258</v>
@@ -4271,7 +4277,7 @@
         <v>42373</v>
       </c>
       <c r="F74" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="G74">
         <v>30960</v>
@@ -4283,10 +4289,10 @@
         <v>93.101300133241523</v>
       </c>
       <c r="J74" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K74" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L74">
         <v>174866.58596225959</v>
@@ -4300,13 +4306,13 @@
     </row>
     <row r="75" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B75">
         <v>1546</v>
       </c>
       <c r="C75" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D75">
         <v>290</v>
@@ -4315,7 +4321,7 @@
         <v>43469</v>
       </c>
       <c r="F75" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G75">
         <v>34800</v>
@@ -4327,10 +4333,10 @@
         <v>95.085951902966272</v>
       </c>
       <c r="J75" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K75" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L75">
         <v>200745.46165754239</v>
@@ -4344,13 +4350,13 @@
     </row>
     <row r="76" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B76">
         <v>1180</v>
       </c>
       <c r="C76" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D76">
         <v>25</v>
@@ -4359,7 +4365,7 @@
         <v>42824</v>
       </c>
       <c r="F76" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G76">
         <v>3000</v>
@@ -4371,10 +4377,10 @@
         <v>93.912911440087655</v>
       </c>
       <c r="J76" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K76" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L76">
         <v>17092.14988209595</v>
@@ -4388,13 +4394,13 @@
     </row>
     <row r="77" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B77">
         <v>1677</v>
       </c>
       <c r="C77" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D77">
         <v>30</v>
@@ -4403,7 +4409,7 @@
         <v>43311</v>
       </c>
       <c r="F77" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="G77">
         <v>3600</v>
@@ -4415,10 +4421,10 @@
         <v>94.797254437211279</v>
       </c>
       <c r="J77" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K77" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L77">
         <v>20703.720369086939</v>
@@ -4432,13 +4438,13 @@
     </row>
     <row r="78" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B78">
         <v>3562</v>
       </c>
       <c r="C78" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D78">
         <v>15</v>
@@ -4447,7 +4453,7 @@
         <v>43537</v>
       </c>
       <c r="F78" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G78">
         <v>1800</v>
@@ -4459,10 +4465,10 @@
         <v>95.210471911057198</v>
       </c>
       <c r="J78" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K78" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L78">
         <v>10396.983532687451</v>
@@ -4476,13 +4482,13 @@
     </row>
     <row r="79" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B79">
         <v>1424</v>
       </c>
       <c r="C79" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D79">
         <v>200</v>
@@ -4491,7 +4497,7 @@
         <v>45138</v>
       </c>
       <c r="F79" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G79">
         <v>24000</v>
@@ -4503,10 +4509,10 @@
         <v>99</v>
       </c>
       <c r="J79" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K79" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L79">
         <v>144144</v>
@@ -4520,13 +4526,13 @@
     </row>
     <row r="80" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B80">
         <v>1410</v>
       </c>
       <c r="C80" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D80">
         <v>245</v>
@@ -4535,7 +4541,7 @@
         <v>43834</v>
       </c>
       <c r="F80" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G80">
         <v>29400</v>
@@ -4547,10 +4553,10 @@
         <v>95.756245622322524</v>
       </c>
       <c r="J80" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K80" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L80">
         <v>170790.83969197451</v>
@@ -4564,13 +4570,13 @@
     </row>
     <row r="81" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B81">
         <v>1775</v>
       </c>
       <c r="C81" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D81">
         <v>93.76</v>
@@ -4579,7 +4585,7 @@
         <v>43467</v>
       </c>
       <c r="F81" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G81">
         <v>11251.2</v>
@@ -4591,10 +4597,10 @@
         <v>95.082292016153659</v>
       </c>
       <c r="J81" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K81" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L81">
         <v>64900.586291883643</v>
@@ -4608,13 +4614,13 @@
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B82">
         <v>1412</v>
       </c>
       <c r="C82" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D82">
         <v>59</v>
@@ -4623,7 +4629,7 @@
         <v>43104</v>
       </c>
       <c r="F82" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="G82">
         <v>7080</v>
@@ -4635,10 +4641,10 @@
         <v>94.420350239645515</v>
       </c>
       <c r="J82" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K82" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L82">
         <v>40555.428834932543</v>
@@ -4652,13 +4658,13 @@
     </row>
     <row r="83" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B83">
         <v>1973</v>
       </c>
       <c r="C83" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D83">
         <v>20</v>
@@ -4667,7 +4673,7 @@
         <v>43109</v>
       </c>
       <c r="F83" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G83">
         <v>2400</v>
@@ -4679,10 +4685,10 @@
         <v>94.429436520685883</v>
       </c>
       <c r="J83" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K83" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L83">
         <v>13748.92595741187</v>
@@ -4696,13 +4702,13 @@
     </row>
     <row r="84" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B84">
         <v>1973</v>
       </c>
       <c r="C84" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D84">
         <v>20</v>
@@ -4711,7 +4717,7 @@
         <v>43762</v>
       </c>
       <c r="F84" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G84">
         <v>2400</v>
@@ -4723,10 +4729,10 @@
         <v>95.623650238871392</v>
       </c>
       <c r="J84" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K84" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L84">
         <v>13922.80347477967</v>
@@ -4740,13 +4746,13 @@
     </row>
     <row r="85" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B85">
         <v>1742</v>
       </c>
       <c r="C85" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D85">
         <v>150</v>
@@ -4755,7 +4761,7 @@
         <v>43843</v>
       </c>
       <c r="F85" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G85">
         <v>18000</v>
@@ -4767,10 +4773,10 @@
         <v>95.772832967811127</v>
       </c>
       <c r="J85" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K85" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L85">
         <v>104583.9336008497</v>
@@ -4784,13 +4790,13 @@
     </row>
     <row r="86" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B86">
         <v>1742</v>
       </c>
       <c r="C86" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D86">
         <v>225</v>
@@ -4799,7 +4805,7 @@
         <v>45231</v>
       </c>
       <c r="F86" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G86">
         <v>27000</v>
@@ -4811,10 +4817,10 @@
         <v>99</v>
       </c>
       <c r="J86" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K86" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L86">
         <v>162162</v>
@@ -4828,13 +4834,13 @@
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B87">
         <v>1588</v>
       </c>
       <c r="C87" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D87">
         <v>12.5</v>
@@ -4843,7 +4849,7 @@
         <v>43160</v>
       </c>
       <c r="F87" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="G87">
         <v>1500</v>
@@ -4855,10 +4861,10 @@
         <v>94.522166547374269</v>
       </c>
       <c r="J87" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K87" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L87">
         <v>8601.5171558110578</v>
@@ -4872,13 +4878,13 @@
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B88">
         <v>1424</v>
       </c>
       <c r="C88" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D88">
         <v>25</v>
@@ -4887,7 +4893,7 @@
         <v>43468</v>
       </c>
       <c r="F88" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="G88">
         <v>3000</v>
@@ -4899,10 +4905,10 @@
         <v>95.084121941950855</v>
       </c>
       <c r="J88" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K88" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L88">
         <v>17305.31019343506</v>
@@ -4916,13 +4922,13 @@
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B89">
         <v>1584</v>
       </c>
       <c r="C89" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D89">
         <v>35</v>
@@ -4931,7 +4937,7 @@
         <v>43543</v>
       </c>
       <c r="F89" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="G89">
         <v>4200</v>
@@ -4943,10 +4949,10 @@
         <v>95.221466796314445</v>
       </c>
       <c r="J89" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K89" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L89">
         <v>24262.429739700921</v>
@@ -4960,13 +4966,13 @@
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B90">
         <v>1164</v>
       </c>
       <c r="C90" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D90">
         <v>123</v>
@@ -4975,7 +4981,7 @@
         <v>43522</v>
       </c>
       <c r="F90" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="G90">
         <v>14760</v>
@@ -4987,10 +4993,10 @@
         <v>95.182990251832777</v>
       </c>
       <c r="J90" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K90" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L90">
         <v>85230.656791101137</v>
@@ -5004,13 +5010,13 @@
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B91">
         <v>1164</v>
       </c>
       <c r="C91" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="D91">
         <v>230</v>
@@ -5019,7 +5025,7 @@
         <v>45016</v>
       </c>
       <c r="F91" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G91">
         <v>27600</v>
@@ -5031,10 +5037,10 @@
         <v>99</v>
       </c>
       <c r="J91" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K91" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L91">
         <v>165765.6</v>
@@ -5048,13 +5054,13 @@
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B92">
         <v>1650</v>
       </c>
       <c r="C92" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D92">
         <v>90</v>
@@ -5063,7 +5069,7 @@
         <v>43434</v>
       </c>
       <c r="F92" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G92">
         <v>10800</v>
@@ -5075,10 +5081,10 @@
         <v>95.021924217828101</v>
       </c>
       <c r="J92" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K92" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L92">
         <v>62258.364747520973</v>
@@ -5092,71 +5098,71 @@
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B93">
         <v>1856</v>
       </c>
       <c r="C93" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D93">
         <v>250</v>
       </c>
       <c r="E93" t="s">
+        <v>189</v>
+      </c>
+      <c r="F93" t="s">
         <v>190</v>
-      </c>
-      <c r="F93" t="s">
-        <v>191</v>
       </c>
       <c r="G93">
         <v>30000</v>
       </c>
       <c r="J93" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K93" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B94">
         <v>1584</v>
       </c>
       <c r="C94" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D94">
         <v>90</v>
       </c>
       <c r="E94" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F94" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G94">
         <v>10800</v>
       </c>
       <c r="J94" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K94" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B95">
         <v>1435</v>
       </c>
       <c r="C95" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D95">
         <v>30</v>
@@ -5165,7 +5171,7 @@
         <v>45747</v>
       </c>
       <c r="F95" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G95">
         <v>3600</v>
@@ -5177,10 +5183,10 @@
         <v>99</v>
       </c>
       <c r="J95" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K95" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L95">
         <v>21621.599999999999</v>
@@ -5188,13 +5194,13 @@
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B96">
         <v>1457</v>
       </c>
       <c r="C96" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D96">
         <v>160</v>
@@ -5203,7 +5209,7 @@
         <v>45747</v>
       </c>
       <c r="F96" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G96">
         <v>19200</v>
@@ -5215,10 +5221,10 @@
         <v>99</v>
       </c>
       <c r="J96" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K96" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L96">
         <v>115315.2</v>
@@ -5226,42 +5232,42 @@
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B97">
         <v>1292</v>
       </c>
       <c r="C97" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D97">
         <v>360</v>
       </c>
       <c r="E97" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F97" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="G97">
         <v>43200</v>
       </c>
       <c r="J97" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K97" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B98">
         <v>1397</v>
       </c>
       <c r="C98" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D98">
         <v>285</v>
@@ -5270,7 +5276,7 @@
         <v>43841</v>
       </c>
       <c r="F98" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G98">
         <v>34200</v>
@@ -5282,10 +5288,10 @@
         <v>95.769146642740267</v>
       </c>
       <c r="J98" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K98" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L98">
         <v>198701.82545435749</v>
@@ -5299,13 +5305,13 @@
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B99">
         <v>1528</v>
       </c>
       <c r="C99" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="D99">
         <v>500</v>
@@ -5314,7 +5320,7 @@
         <v>45838</v>
       </c>
       <c r="F99" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G99">
         <v>60000</v>
@@ -5326,10 +5332,10 @@
         <v>99</v>
       </c>
       <c r="J99" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K99" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L99">
         <v>360360</v>
@@ -5343,13 +5349,13 @@
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B100">
         <v>1436</v>
       </c>
       <c r="C100" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D100">
         <v>25</v>
@@ -5358,7 +5364,7 @@
         <v>45747</v>
       </c>
       <c r="F100" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G100">
         <v>3000</v>
@@ -5370,10 +5376,10 @@
         <v>99</v>
       </c>
       <c r="J100" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K100" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L100">
         <v>18018</v>
@@ -5387,13 +5393,13 @@
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B101">
         <v>1180</v>
       </c>
       <c r="C101" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D101">
         <v>120</v>
@@ -5402,7 +5408,7 @@
         <v>43553</v>
       </c>
       <c r="F101" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G101">
         <v>14400</v>
@@ -5414,10 +5420,10 @@
         <v>95.239794426675687</v>
       </c>
       <c r="J101" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K101" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L101">
         <v>83201.484411143887</v>
@@ -5431,13 +5437,13 @@
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B102">
         <v>1587</v>
       </c>
       <c r="C102" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D102">
         <v>0</v>
@@ -5446,7 +5452,7 @@
         <v>43504</v>
       </c>
       <c r="F102" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G102">
         <v>0</v>
@@ -5458,10 +5464,10 @@
         <v>95.150022731247432</v>
       </c>
       <c r="J102" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K102" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="L102">
         <v>0</v>
@@ -5469,60 +5475,60 @@
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B103">
         <v>1259</v>
       </c>
       <c r="C103" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D103">
         <v>200</v>
       </c>
       <c r="E103" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F103" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G103">
         <v>24000</v>
       </c>
       <c r="J103" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="K103" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B104">
         <v>1937</v>
       </c>
       <c r="C104" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D104">
         <v>400</v>
       </c>
       <c r="E104" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F104" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G104">
         <v>48000</v>
       </c>
       <c r="J104" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K104" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update column name from 'Plant Capacity  KWp' to 'Plant Capacity'
</commit_message>
<xml_diff>
--- a/orchestrator/masters/Solar_installation.xlsx
+++ b/orchestrator/masters/Solar_installation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/HPCL_INFRA/dnc_backend_v2/orchestrator/masters/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8587A661-732C-8945-92AA-E6ECC1724000}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39B1D71-375B-EA44-BE2D-0D7EF6549B2A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -655,7 +655,7 @@
     <t>1937/Suryapet Terminal/400KWp/Set-2</t>
   </si>
   <si>
-    <t>Plant Capacity  KWp</t>
+    <t>Plant Capacity</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Update Solar_installation.xlsx master file
</commit_message>
<xml_diff>
--- a/orchestrator/masters/Solar_installation.xlsx
+++ b/orchestrator/masters/Solar_installation.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Documents/HPCL_INFRA/dnc_backend_v2/orchestrator/masters/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/apple/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39B1D71-375B-EA44-BE2D-0D7EF6549B2A}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36CF5AAE-3F67-524C-9621-D9C2ADDD03FF}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="534" uniqueCount="212">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="212">
   <si>
     <t>Zone</t>
   </si>
@@ -677,6 +677,7 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
@@ -1029,7 +1030,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N104"/>
+  <dimension ref="A1:N105"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.6640625" bestFit="1" customWidth="1"/>
@@ -5531,6 +5532,32 @@
         <v>17</v>
       </c>
     </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>60</v>
+      </c>
+      <c r="B105">
+        <v>1650</v>
+      </c>
+      <c r="C105" t="s">
+        <v>187</v>
+      </c>
+      <c r="D105">
+        <v>90</v>
+      </c>
+      <c r="E105" s="2">
+        <v>45747</v>
+      </c>
+      <c r="G105">
+        <v>10800</v>
+      </c>
+      <c r="J105" t="s">
+        <v>24</v>
+      </c>
+      <c r="K105" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>